<commit_message>
Completed SauceDemo Manual Testing Portfolio
</commit_message>
<xml_diff>
--- a/Project-01-Ecommerce-Manual-Testing/Test senarios/login test scenarios.xlsx
+++ b/Project-01-Ecommerce-Manual-Testing/Test senarios/login test scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yashwanth y v\Desktop\QA portfolio\Project-01-Ecommerce-Manual-Testing\Test senarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A781A5E7-0524-48E2-B5FD-5D43469FAD62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8082567C-F0E3-4A8C-A136-12AF130148CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>Scenario ID</t>
   </si>
   <si>
-    <t>Module</t>
-  </si>
-  <si>
     <t>Test Scenario</t>
   </si>
   <si>
@@ -42,9 +39,6 @@
     <t>TS001</t>
   </si>
   <si>
-    <t>Login</t>
-  </si>
-  <si>
     <t>Verify login with valid username and valid password.</t>
   </si>
   <si>
@@ -90,85 +84,22 @@
     <t>TS008</t>
   </si>
   <si>
-    <t>Verify login using only spaces in the username field.</t>
-  </si>
-  <si>
     <t>Medium</t>
   </si>
   <si>
     <t>TS009</t>
   </si>
   <si>
-    <t>Verify login using only spaces in the password field.</t>
-  </si>
-  <si>
     <t>TS010</t>
   </si>
   <si>
-    <t>Verify the error message for invalid credentials.</t>
-  </si>
-  <si>
-    <t>TS011</t>
-  </si>
-  <si>
     <t>Verify the password field masks entered characters.</t>
   </si>
   <si>
-    <t>TS012</t>
-  </si>
-  <si>
     <t>Verify successful login redirects to the Products page.</t>
   </si>
   <si>
-    <t>TS013</t>
-  </si>
-  <si>
-    <t>Verify the Login button is clickable.</t>
-  </si>
-  <si>
-    <t>TS014</t>
-  </si>
-  <si>
     <t>Verify the application behavior using the locked user account.</t>
-  </si>
-  <si>
-    <t>TS015</t>
-  </si>
-  <si>
-    <t>Verify login after refreshing the page.</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>TS016</t>
-  </si>
-  <si>
-    <t>Verify login using copied and pasted credentials.</t>
-  </si>
-  <si>
-    <t>TS017</t>
-  </si>
-  <si>
-    <t>Verify login using keyboard navigation (Tab and Enter).</t>
-  </si>
-  <si>
-    <t>TS018</t>
-  </si>
-  <si>
-    <t>Verify the login page loads successfully.</t>
-  </si>
-  <si>
-    <t>TS019</t>
-  </si>
-  <si>
-    <t>Verify the username and password fields accept input.</t>
-  </si>
-  <si>
-    <t>TS020</t>
-  </si>
-  <si>
-    <t>Verify that users cannot access the Products page without logging in.</t>
   </si>
 </sst>
 </file>
@@ -500,13 +431,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="32.77734375" customWidth="1"/>
+    <col min="2" max="2" width="50.109375" customWidth="1"/>
+    <col min="3" max="3" width="27.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -516,288 +448,115 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="C5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="C8" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="C11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>